<commit_message>
#38 Parts properties changed: Client BOM updated.
</commit_message>
<xml_diff>
--- a/Design Files/IoT-Speaker-v1.4/BOM/Client BOM IoT-Speaker v1.4.xlsx
+++ b/Design Files/IoT-Speaker-v1.4/BOM/Client BOM IoT-Speaker v1.4.xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MarsVirgo\Documents\GitHub\smartmasjid-hardware\Design Files\IoT-Speaker-v1.4\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LiberDB\Documents\GitHub\smartmasjid-hardware\Design Files\IoT-Speaker-v1.4\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="471" uniqueCount="273">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="488" uniqueCount="277">
   <si>
     <t>Component list</t>
   </si>
@@ -781,9 +781,6 @@
     <t>C2, C3, C7, C18, C20, C83</t>
   </si>
   <si>
-    <t>C1, C5, C6, C13, C16</t>
-  </si>
-  <si>
     <t>DNP</t>
   </si>
   <si>
@@ -851,6 +848,21 @@
   </si>
   <si>
     <t>Bill of Materials for Project [IoT-Speaker v1.4]</t>
+  </si>
+  <si>
+    <t>C1, C5, C6, C16</t>
+  </si>
+  <si>
+    <t>LED1</t>
+  </si>
+  <si>
+    <t>R29, R31, R34, R36, R37, R38</t>
+  </si>
+  <si>
+    <t>Emerald 0603 Light Emitting Diodes (LED) ROHS</t>
+  </si>
+  <si>
+    <t>NCD0603G2</t>
   </si>
 </sst>
 </file>
@@ -1037,7 +1049,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1062,6 +1074,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD3D3D3"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="27">
     <border>
@@ -1380,7 +1398,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="85">
+  <cellXfs count="88">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1549,6 +1567,45 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="3" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1576,44 +1633,14 @@
     <xf numFmtId="0" fontId="17" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="3" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="3" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1948,7 +1975,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:M73"/>
+  <dimension ref="A1:O75"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="1" customWidth="1"/>
@@ -1963,9 +1990,10 @@
     <col min="11" max="11" width="8.7109375" customWidth="1"/>
     <col min="12" max="12" width="18.28515625" customWidth="1"/>
     <col min="13" max="13" width="29.42578125" customWidth="1"/>
+    <col min="15" max="15" width="23.28515625" style="85" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:15">
       <c r="A1" s="2"/>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -1974,13 +2002,14 @@
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
       <c r="H1" s="4"/>
-      <c r="I1" s="63"/>
-      <c r="J1" s="63"/>
-      <c r="K1" s="63"/>
-      <c r="L1" s="63"/>
-      <c r="M1" s="63"/>
-    </row>
-    <row r="2" spans="1:13" ht="31.5">
+      <c r="I1" s="76"/>
+      <c r="J1" s="76"/>
+      <c r="K1" s="76"/>
+      <c r="L1" s="76"/>
+      <c r="M1" s="76"/>
+      <c r="O1" s="86"/>
+    </row>
+    <row r="2" spans="1:15" ht="31.5">
       <c r="A2" s="2"/>
       <c r="B2" s="5"/>
       <c r="C2" s="6"/>
@@ -1988,8 +2017,8 @@
         <v>0</v>
       </c>
       <c r="E2" s="7"/>
-      <c r="F2" s="84" t="s">
-        <v>272</v>
+      <c r="F2" s="75" t="s">
+        <v>271</v>
       </c>
       <c r="G2" s="8"/>
       <c r="H2" s="9"/>
@@ -1998,8 +2027,9 @@
       <c r="K2" s="9"/>
       <c r="L2" s="9"/>
       <c r="M2" s="54"/>
-    </row>
-    <row r="3" spans="1:13">
+      <c r="O2" s="87"/>
+    </row>
+    <row r="3" spans="1:15">
       <c r="A3" s="2"/>
       <c r="B3" s="10"/>
       <c r="C3" s="11"/>
@@ -2007,8 +2037,8 @@
         <v>1</v>
       </c>
       <c r="E3" s="12"/>
-      <c r="F3" s="83" t="s">
-        <v>271</v>
+      <c r="F3" s="74" t="s">
+        <v>270</v>
       </c>
       <c r="G3" s="12"/>
       <c r="H3" s="13"/>
@@ -2016,9 +2046,10 @@
       <c r="J3" s="13"/>
       <c r="K3" s="13"/>
       <c r="L3" s="13"/>
-      <c r="M3" s="64"/>
-    </row>
-    <row r="4" spans="1:13">
+      <c r="M3" s="77"/>
+      <c r="O3" s="87"/>
+    </row>
+    <row r="4" spans="1:15">
       <c r="A4" s="2"/>
       <c r="B4" s="10"/>
       <c r="C4" s="11"/>
@@ -2026,8 +2057,8 @@
         <v>2</v>
       </c>
       <c r="E4" s="12"/>
-      <c r="F4" s="83" t="s">
-        <v>271</v>
+      <c r="F4" s="74" t="s">
+        <v>270</v>
       </c>
       <c r="G4" s="14"/>
       <c r="H4" s="15"/>
@@ -2035,9 +2066,10 @@
       <c r="J4" s="15"/>
       <c r="K4" s="15"/>
       <c r="L4" s="15"/>
-      <c r="M4" s="65"/>
-    </row>
-    <row r="5" spans="1:13">
+      <c r="M4" s="78"/>
+      <c r="O4" s="87"/>
+    </row>
+    <row r="5" spans="1:15">
       <c r="A5" s="2"/>
       <c r="B5" s="10"/>
       <c r="C5" s="11"/>
@@ -2054,9 +2086,10 @@
       <c r="J5" s="17"/>
       <c r="K5" s="17"/>
       <c r="L5" s="17"/>
-      <c r="M5" s="65"/>
-    </row>
-    <row r="6" spans="1:13">
+      <c r="M5" s="78"/>
+      <c r="O5" s="87"/>
+    </row>
+    <row r="6" spans="1:15">
       <c r="A6" s="2"/>
       <c r="B6" s="18"/>
       <c r="C6" s="19"/>
@@ -2069,9 +2102,10 @@
       <c r="J6" s="17"/>
       <c r="K6" s="17"/>
       <c r="L6" s="17"/>
-      <c r="M6" s="65"/>
-    </row>
-    <row r="7" spans="1:13">
+      <c r="M6" s="78"/>
+      <c r="O6" s="87"/>
+    </row>
+    <row r="7" spans="1:15">
       <c r="A7" s="2"/>
       <c r="B7" s="22"/>
       <c r="C7" s="23"/>
@@ -2084,9 +2118,10 @@
       <c r="J7" s="26"/>
       <c r="K7" s="26"/>
       <c r="L7" s="26"/>
-      <c r="M7" s="65"/>
-    </row>
-    <row r="8" spans="1:13">
+      <c r="M7" s="78"/>
+      <c r="O7" s="87"/>
+    </row>
+    <row r="8" spans="1:15">
       <c r="A8" s="2"/>
       <c r="B8" s="27"/>
       <c r="C8" s="28"/>
@@ -2099,9 +2134,10 @@
       <c r="J8" s="26"/>
       <c r="K8" s="26"/>
       <c r="L8" s="26"/>
-      <c r="M8" s="65"/>
-    </row>
-    <row r="9" spans="1:13">
+      <c r="M8" s="78"/>
+      <c r="O8" s="87"/>
+    </row>
+    <row r="9" spans="1:15">
       <c r="A9" s="2"/>
       <c r="B9" s="31" t="s">
         <v>5</v>
@@ -2139,8 +2175,9 @@
       <c r="M9" s="31" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="10" spans="1:13">
+      <c r="O9" s="87"/>
+    </row>
+    <row r="10" spans="1:15">
       <c r="A10" s="2"/>
       <c r="B10" s="34">
         <f>ROW(B10)-ROW($B$9)</f>
@@ -2149,8 +2186,8 @@
       <c r="C10" s="35" t="s">
         <v>17</v>
       </c>
-      <c r="D10" s="72" t="s">
-        <v>249</v>
+      <c r="D10" s="63" t="s">
+        <v>272</v>
       </c>
       <c r="E10" s="37" t="s">
         <v>18</v>
@@ -2169,26 +2206,27 @@
       </c>
       <c r="J10" s="36"/>
       <c r="K10" s="56">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L10" s="37">
         <f>K10*5</f>
-        <v>25</v>
-      </c>
-      <c r="M10" s="73" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13">
+        <v>20</v>
+      </c>
+      <c r="M10" s="64" t="s">
+        <v>249</v>
+      </c>
+      <c r="O10" s="87"/>
+    </row>
+    <row r="11" spans="1:15">
       <c r="A11" s="2"/>
       <c r="B11" s="34">
-        <f t="shared" ref="B11:B71" si="0">ROW(B11)-ROW($B$9)</f>
+        <f t="shared" ref="B11:B73" si="0">ROW(B11)-ROW($B$9)</f>
         <v>2</v>
       </c>
       <c r="C11" s="35" t="s">
         <v>17</v>
       </c>
-      <c r="D11" s="82" t="s">
+      <c r="D11" s="73" t="s">
         <v>248</v>
       </c>
       <c r="E11" s="40" t="s">
@@ -2214,11 +2252,12 @@
         <f t="shared" ref="L11:L13" si="1">K11*5</f>
         <v>30</v>
       </c>
-      <c r="M11" s="74" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13" ht="15.75" thickBot="1">
+      <c r="M11" s="65" t="s">
+        <v>249</v>
+      </c>
+      <c r="O11" s="87"/>
+    </row>
+    <row r="12" spans="1:15" ht="15.75" thickBot="1">
       <c r="A12" s="2"/>
       <c r="B12" s="34">
         <f t="shared" si="0"/>
@@ -2227,7 +2266,7 @@
       <c r="C12" s="35" t="s">
         <v>17</v>
       </c>
-      <c r="D12" s="72" t="s">
+      <c r="D12" s="63" t="s">
         <v>27</v>
       </c>
       <c r="E12" s="37" t="s">
@@ -2254,8 +2293,9 @@
         <v>15</v>
       </c>
       <c r="M12" s="36"/>
-    </row>
-    <row r="13" spans="1:13" ht="15.75" thickBot="1">
+      <c r="O12" s="87"/>
+    </row>
+    <row r="13" spans="1:15" ht="15.75" thickBot="1">
       <c r="A13" s="2"/>
       <c r="B13" s="34">
         <f t="shared" si="0"/>
@@ -2264,7 +2304,7 @@
       <c r="C13" s="35" t="s">
         <v>17</v>
       </c>
-      <c r="D13" s="82" t="s">
+      <c r="D13" s="73" t="s">
         <v>247</v>
       </c>
       <c r="E13" s="37" t="s">
@@ -2291,8 +2331,9 @@
         <v>40</v>
       </c>
       <c r="M13" s="36"/>
-    </row>
-    <row r="14" spans="1:13" ht="15.75" thickBot="1">
+      <c r="O13" s="87"/>
+    </row>
+    <row r="14" spans="1:15" ht="15.75" thickBot="1">
       <c r="A14" s="2"/>
       <c r="B14" s="34">
         <f t="shared" si="0"/>
@@ -2301,7 +2342,7 @@
       <c r="C14" s="35" t="s">
         <v>17</v>
       </c>
-      <c r="D14" s="82" t="s">
+      <c r="D14" s="73" t="s">
         <v>32</v>
       </c>
       <c r="E14" s="40" t="s">
@@ -2328,8 +2369,9 @@
         <v>10</v>
       </c>
       <c r="M14" s="39"/>
-    </row>
-    <row r="15" spans="1:13" ht="15.75" thickBot="1">
+      <c r="O14" s="87"/>
+    </row>
+    <row r="15" spans="1:15" ht="15.75" thickBot="1">
       <c r="A15" s="2"/>
       <c r="B15" s="34">
         <f t="shared" si="0"/>
@@ -2338,8 +2380,8 @@
       <c r="C15" s="35" t="s">
         <v>17</v>
       </c>
-      <c r="D15" s="82" t="s">
-        <v>251</v>
+      <c r="D15" s="73" t="s">
+        <v>250</v>
       </c>
       <c r="E15" s="40" t="s">
         <v>18</v>
@@ -2365,8 +2407,9 @@
         <v>10</v>
       </c>
       <c r="M15" s="36"/>
-    </row>
-    <row r="16" spans="1:13" ht="15.75" thickBot="1">
+      <c r="O15" s="87"/>
+    </row>
+    <row r="16" spans="1:15" ht="15.75" thickBot="1">
       <c r="A16" s="2"/>
       <c r="B16" s="34">
         <f t="shared" si="0"/>
@@ -2375,8 +2418,8 @@
       <c r="C16" s="35" t="s">
         <v>17</v>
       </c>
-      <c r="D16" s="77" t="s">
-        <v>252</v>
+      <c r="D16" s="68" t="s">
+        <v>251</v>
       </c>
       <c r="E16" s="37" t="s">
         <v>36</v>
@@ -2402,8 +2445,9 @@
         <v>15</v>
       </c>
       <c r="M16" s="36"/>
-    </row>
-    <row r="17" spans="1:13" ht="15.75" thickBot="1">
+      <c r="O16" s="87"/>
+    </row>
+    <row r="17" spans="1:15" ht="15.75" thickBot="1">
       <c r="A17" s="2"/>
       <c r="B17" s="34">
         <f t="shared" si="0"/>
@@ -2412,8 +2456,8 @@
       <c r="C17" s="35" t="s">
         <v>17</v>
       </c>
-      <c r="D17" s="78" t="s">
-        <v>253</v>
+      <c r="D17" s="69" t="s">
+        <v>252</v>
       </c>
       <c r="E17" s="40" t="s">
         <v>39</v>
@@ -2439,8 +2483,9 @@
         <v>10</v>
       </c>
       <c r="M17" s="39"/>
-    </row>
-    <row r="18" spans="1:13" ht="15.75" thickBot="1">
+      <c r="O17" s="87"/>
+    </row>
+    <row r="18" spans="1:15" ht="15.75" thickBot="1">
       <c r="A18" s="2"/>
       <c r="B18" s="34">
         <f t="shared" si="0"/>
@@ -2449,16 +2494,16 @@
       <c r="C18" s="35" t="s">
         <v>17</v>
       </c>
-      <c r="D18" s="77" t="s">
-        <v>255</v>
-      </c>
-      <c r="E18" s="79" t="s">
+      <c r="D18" s="68" t="s">
+        <v>254</v>
+      </c>
+      <c r="E18" s="70" t="s">
         <v>39</v>
       </c>
-      <c r="F18" s="76" t="s">
+      <c r="F18" s="67" t="s">
         <v>29</v>
       </c>
-      <c r="G18" s="80" t="s">
+      <c r="G18" s="71" t="s">
         <v>40</v>
       </c>
       <c r="H18" s="40" t="s">
@@ -2475,11 +2520,12 @@
         <f t="shared" si="3"/>
         <v>10</v>
       </c>
-      <c r="M18" s="73" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="19" spans="1:13" ht="15.75" thickBot="1">
+      <c r="M18" s="64" t="s">
+        <v>249</v>
+      </c>
+      <c r="O18" s="87"/>
+    </row>
+    <row r="19" spans="1:15" ht="15.75" thickBot="1">
       <c r="A19" s="2"/>
       <c r="B19" s="34">
         <f t="shared" si="0"/>
@@ -2488,16 +2534,16 @@
       <c r="C19" s="35" t="s">
         <v>17</v>
       </c>
-      <c r="D19" s="78" t="s">
-        <v>254</v>
+      <c r="D19" s="69" t="s">
+        <v>253</v>
       </c>
       <c r="E19" s="40" t="s">
         <v>36</v>
       </c>
-      <c r="F19" s="76" t="s">
+      <c r="F19" s="67" t="s">
         <v>29</v>
       </c>
-      <c r="G19" s="80" t="s">
+      <c r="G19" s="71" t="s">
         <v>37</v>
       </c>
       <c r="H19" s="40" t="s">
@@ -2514,11 +2560,12 @@
         <f t="shared" si="3"/>
         <v>5</v>
       </c>
-      <c r="M19" s="73" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="20" spans="1:13" ht="15.75" thickBot="1">
+      <c r="M19" s="64" t="s">
+        <v>249</v>
+      </c>
+      <c r="O19" s="87"/>
+    </row>
+    <row r="20" spans="1:15" ht="15.75" thickBot="1">
       <c r="A20" s="2"/>
       <c r="B20" s="34">
         <f t="shared" si="0"/>
@@ -2527,7 +2574,7 @@
       <c r="C20" s="42" t="s">
         <v>17</v>
       </c>
-      <c r="D20" s="77" t="s">
+      <c r="D20" s="68" t="s">
         <v>42</v>
       </c>
       <c r="E20" s="36" t="s">
@@ -2554,8 +2601,9 @@
         <v>5</v>
       </c>
       <c r="M20" s="36"/>
-    </row>
-    <row r="21" spans="1:13">
+      <c r="O20" s="87"/>
+    </row>
+    <row r="21" spans="1:15">
       <c r="A21" s="2"/>
       <c r="B21" s="34">
         <f t="shared" si="0"/>
@@ -2564,7 +2612,7 @@
       <c r="C21" s="43" t="s">
         <v>47</v>
       </c>
-      <c r="D21" s="77" t="s">
+      <c r="D21" s="68" t="s">
         <v>48</v>
       </c>
       <c r="E21" s="37" t="s">
@@ -2591,8 +2639,9 @@
         <v>5</v>
       </c>
       <c r="M21" s="36"/>
-    </row>
-    <row r="22" spans="1:13" ht="24">
+      <c r="O21" s="87"/>
+    </row>
+    <row r="22" spans="1:15" ht="24">
       <c r="A22" s="2"/>
       <c r="B22" s="34">
         <f t="shared" si="0"/>
@@ -2601,7 +2650,7 @@
       <c r="C22" s="43" t="s">
         <v>47</v>
       </c>
-      <c r="D22" s="77" t="s">
+      <c r="D22" s="68" t="s">
         <v>54</v>
       </c>
       <c r="E22" s="40" t="s">
@@ -2627,11 +2676,12 @@
         <f t="shared" ref="L22:L23" si="4">K22*5</f>
         <v>5</v>
       </c>
-      <c r="M22" s="73" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="23" spans="1:13" ht="24">
+      <c r="M22" s="64" t="s">
+        <v>249</v>
+      </c>
+      <c r="O22" s="87"/>
+    </row>
+    <row r="23" spans="1:15" ht="24">
       <c r="A23" s="2"/>
       <c r="B23" s="34">
         <f t="shared" si="0"/>
@@ -2640,7 +2690,7 @@
       <c r="C23" s="43" t="s">
         <v>59</v>
       </c>
-      <c r="D23" s="77" t="s">
+      <c r="D23" s="68" t="s">
         <v>60</v>
       </c>
       <c r="E23" s="37" t="s">
@@ -2667,8 +2717,9 @@
         <v>5</v>
       </c>
       <c r="M23" s="36"/>
-    </row>
-    <row r="24" spans="1:13" ht="36">
+      <c r="O23" s="87"/>
+    </row>
+    <row r="24" spans="1:15" ht="36">
       <c r="A24" s="2"/>
       <c r="B24" s="34">
         <f t="shared" si="0"/>
@@ -2677,7 +2728,7 @@
       <c r="C24" s="35" t="s">
         <v>65</v>
       </c>
-      <c r="D24" s="77" t="s">
+      <c r="D24" s="68" t="s">
         <v>66</v>
       </c>
       <c r="E24" s="40" t="s">
@@ -2704,8 +2755,9 @@
         <v>15</v>
       </c>
       <c r="M24" s="39"/>
-    </row>
-    <row r="25" spans="1:13">
+      <c r="O24" s="87"/>
+    </row>
+    <row r="25" spans="1:15">
       <c r="A25" s="2"/>
       <c r="B25" s="34">
         <f t="shared" si="0"/>
@@ -2714,7 +2766,7 @@
       <c r="C25" s="43" t="s">
         <v>65</v>
       </c>
-      <c r="D25" s="72" t="s">
+      <c r="D25" s="63" t="s">
         <v>71</v>
       </c>
       <c r="E25" s="37" t="s">
@@ -2741,8 +2793,9 @@
         <v>5</v>
       </c>
       <c r="M25" s="36"/>
-    </row>
-    <row r="26" spans="1:13" ht="36">
+      <c r="O25" s="87"/>
+    </row>
+    <row r="26" spans="1:15" ht="36">
       <c r="A26" s="2"/>
       <c r="B26" s="34">
         <f t="shared" si="0"/>
@@ -2751,7 +2804,7 @@
       <c r="C26" s="35" t="s">
         <v>75</v>
       </c>
-      <c r="D26" s="82" t="s">
+      <c r="D26" s="73" t="s">
         <v>76</v>
       </c>
       <c r="E26" s="40" t="s">
@@ -2777,11 +2830,12 @@
         <f t="shared" ref="L26:L27" si="6">K26*5</f>
         <v>5</v>
       </c>
-      <c r="M26" s="73" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="27" spans="1:13" ht="24">
+      <c r="M26" s="64" t="s">
+        <v>249</v>
+      </c>
+      <c r="O26" s="87"/>
+    </row>
+    <row r="27" spans="1:15" ht="24">
       <c r="A27" s="2"/>
       <c r="B27" s="34">
         <f t="shared" si="0"/>
@@ -2790,7 +2844,7 @@
       <c r="C27" s="43" t="s">
         <v>81</v>
       </c>
-      <c r="D27" s="72" t="s">
+      <c r="D27" s="63" t="s">
         <v>82</v>
       </c>
       <c r="E27" s="37" t="s">
@@ -2817,8 +2871,9 @@
         <v>5</v>
       </c>
       <c r="M27" s="36"/>
-    </row>
-    <row r="28" spans="1:13" ht="36">
+      <c r="O27" s="87"/>
+    </row>
+    <row r="28" spans="1:15" ht="36">
       <c r="A28" s="2"/>
       <c r="B28" s="34">
         <f t="shared" si="0"/>
@@ -2827,7 +2882,7 @@
       <c r="C28" s="35" t="s">
         <v>87</v>
       </c>
-      <c r="D28" s="82" t="s">
+      <c r="D28" s="73" t="s">
         <v>88</v>
       </c>
       <c r="E28" s="40" t="s">
@@ -2854,8 +2909,9 @@
         <v>5</v>
       </c>
       <c r="M28" s="39"/>
-    </row>
-    <row r="29" spans="1:13">
+      <c r="O28" s="87"/>
+    </row>
+    <row r="29" spans="1:15">
       <c r="A29" s="2"/>
       <c r="B29" s="34">
         <f t="shared" si="0"/>
@@ -2864,7 +2920,7 @@
       <c r="C29" s="43" t="s">
         <v>93</v>
       </c>
-      <c r="D29" s="72" t="s">
+      <c r="D29" s="63" t="s">
         <v>94</v>
       </c>
       <c r="E29" s="37" t="s">
@@ -2891,8 +2947,9 @@
         <v>5</v>
       </c>
       <c r="M29" s="36"/>
-    </row>
-    <row r="30" spans="1:13" ht="24">
+      <c r="O29" s="87"/>
+    </row>
+    <row r="30" spans="1:15" ht="24">
       <c r="A30" s="2"/>
       <c r="B30" s="34">
         <f t="shared" si="0"/>
@@ -2901,7 +2958,7 @@
       <c r="C30" s="35" t="s">
         <v>98</v>
       </c>
-      <c r="D30" s="82" t="s">
+      <c r="D30" s="73" t="s">
         <v>99</v>
       </c>
       <c r="E30" s="40" t="s">
@@ -2924,14 +2981,15 @@
         <v>1</v>
       </c>
       <c r="L30" s="40">
-        <f t="shared" ref="L30:L31" si="8">K30*5</f>
+        <f t="shared" ref="L30:L32" si="8">K30*5</f>
         <v>5</v>
       </c>
-      <c r="M30" s="73" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="31" spans="1:13" ht="24">
+      <c r="M30" s="64" t="s">
+        <v>249</v>
+      </c>
+      <c r="O30" s="87"/>
+    </row>
+    <row r="31" spans="1:15" ht="24.75" thickBot="1">
       <c r="A31" s="2"/>
       <c r="B31" s="34">
         <f t="shared" si="0"/>
@@ -2940,7 +2998,7 @@
       <c r="C31" s="43" t="s">
         <v>104</v>
       </c>
-      <c r="D31" s="72" t="s">
+      <c r="D31" s="63" t="s">
         <v>105</v>
       </c>
       <c r="E31" s="37" t="s">
@@ -2967,8 +3025,9 @@
         <v>10</v>
       </c>
       <c r="M31" s="36"/>
-    </row>
-    <row r="32" spans="1:13" ht="24">
+      <c r="O31" s="87"/>
+    </row>
+    <row r="32" spans="1:15" ht="24.75" thickBot="1">
       <c r="A32" s="2"/>
       <c r="B32" s="34">
         <f t="shared" si="0"/>
@@ -2977,152 +3036,156 @@
       <c r="C32" s="35" t="s">
         <v>110</v>
       </c>
-      <c r="D32" s="82" t="s">
-        <v>111</v>
-      </c>
-      <c r="E32" s="40" t="s">
-        <v>112</v>
+      <c r="D32" s="73" t="s">
+        <v>273</v>
+      </c>
+      <c r="E32" s="37" t="s">
+        <v>275</v>
       </c>
       <c r="F32" s="39" t="s">
         <v>113</v>
       </c>
-      <c r="G32" s="40" t="s">
-        <v>114</v>
+      <c r="G32" s="37" t="s">
+        <v>276</v>
       </c>
       <c r="H32" s="41" t="s">
         <v>115</v>
       </c>
-      <c r="I32" s="39" t="s">
+      <c r="I32" s="36" t="s">
         <v>53</v>
       </c>
-      <c r="J32" s="39"/>
-      <c r="K32" s="57">
+      <c r="J32" s="36"/>
+      <c r="K32" s="56">
         <v>1</v>
       </c>
-      <c r="L32" s="40">
-        <f t="shared" ref="L32:L34" si="9">K32*5</f>
+      <c r="L32" s="37">
+        <f t="shared" si="8"/>
         <v>5</v>
       </c>
-      <c r="M32" s="73" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="33" spans="1:13" ht="24">
+      <c r="M32" s="64" t="s">
+        <v>249</v>
+      </c>
+      <c r="O32" s="87"/>
+    </row>
+    <row r="33" spans="1:15" ht="24.75" thickBot="1">
       <c r="A33" s="2"/>
       <c r="B33" s="34">
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
-      <c r="C33" s="43" t="s">
+      <c r="C33" s="35" t="s">
+        <v>110</v>
+      </c>
+      <c r="D33" s="73" t="s">
+        <v>111</v>
+      </c>
+      <c r="E33" s="40" t="s">
+        <v>112</v>
+      </c>
+      <c r="F33" s="39" t="s">
+        <v>113</v>
+      </c>
+      <c r="G33" s="40" t="s">
+        <v>114</v>
+      </c>
+      <c r="H33" s="41" t="s">
+        <v>115</v>
+      </c>
+      <c r="I33" s="39" t="s">
+        <v>53</v>
+      </c>
+      <c r="J33" s="39"/>
+      <c r="K33" s="57">
+        <v>1</v>
+      </c>
+      <c r="L33" s="40">
+        <f t="shared" ref="L33:L35" si="9">K33*5</f>
+        <v>5</v>
+      </c>
+      <c r="M33" s="64" t="s">
+        <v>249</v>
+      </c>
+      <c r="O33" s="87"/>
+    </row>
+    <row r="34" spans="1:15" ht="24">
+      <c r="A34" s="2"/>
+      <c r="B34" s="34">
+        <f t="shared" si="0"/>
+        <v>25</v>
+      </c>
+      <c r="C34" s="43" t="s">
         <v>116</v>
       </c>
-      <c r="D33" s="72" t="s">
+      <c r="D34" s="63" t="s">
         <v>117</v>
       </c>
-      <c r="E33" s="37" t="s">
+      <c r="E34" s="37" t="s">
         <v>118</v>
       </c>
-      <c r="F33" s="36" t="s">
+      <c r="F34" s="36" t="s">
         <v>119</v>
       </c>
-      <c r="G33" s="37" t="s">
+      <c r="G34" s="37" t="s">
         <v>119</v>
       </c>
-      <c r="H33" s="38" t="s">
+      <c r="H34" s="38" t="s">
         <v>120</v>
       </c>
-      <c r="I33" s="36" t="s">
+      <c r="I34" s="36" t="s">
         <v>53</v>
       </c>
-      <c r="J33" s="36"/>
-      <c r="K33" s="56">
+      <c r="J34" s="36"/>
+      <c r="K34" s="56">
         <v>3</v>
       </c>
-      <c r="L33" s="37">
+      <c r="L34" s="37">
         <f t="shared" si="9"/>
         <v>15</v>
       </c>
-      <c r="M33" s="36"/>
-    </row>
-    <row r="34" spans="1:13" ht="36">
-      <c r="A34" s="2"/>
-      <c r="B34" s="34">
-        <f t="shared" si="0"/>
-        <v>25</v>
-      </c>
-      <c r="C34" s="43" t="s">
+      <c r="M34" s="36"/>
+      <c r="O34" s="87"/>
+    </row>
+    <row r="35" spans="1:15" ht="36">
+      <c r="A35" s="2"/>
+      <c r="B35" s="34">
+        <f t="shared" si="0"/>
+        <v>26</v>
+      </c>
+      <c r="C35" s="43" t="s">
         <v>121</v>
       </c>
-      <c r="D34" s="72" t="s">
+      <c r="D35" s="63" t="s">
         <v>122</v>
       </c>
-      <c r="E34" s="37" t="s">
+      <c r="E35" s="37" t="s">
         <v>123</v>
       </c>
-      <c r="F34" s="36" t="s">
+      <c r="F35" s="36" t="s">
         <v>124</v>
       </c>
-      <c r="G34" s="37" t="s">
+      <c r="G35" s="37" t="s">
         <v>125</v>
       </c>
-      <c r="H34" s="38" t="s">
+      <c r="H35" s="38" t="s">
         <v>126</v>
       </c>
-      <c r="I34" s="36" t="s">
+      <c r="I35" s="36" t="s">
         <v>53</v>
       </c>
-      <c r="J34" s="36"/>
-      <c r="K34" s="56">
+      <c r="J35" s="36"/>
+      <c r="K35" s="56">
         <v>1</v>
       </c>
-      <c r="L34" s="37">
+      <c r="L35" s="37">
         <f t="shared" si="9"/>
         <v>5</v>
       </c>
-      <c r="M34" s="73" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="35" spans="1:13" ht="48.75" thickBot="1">
-      <c r="A35" s="2"/>
-      <c r="B35" s="34">
-        <f t="shared" si="0"/>
-        <v>26</v>
-      </c>
-      <c r="C35" s="35" t="s">
-        <v>121</v>
-      </c>
-      <c r="D35" s="78" t="s">
-        <v>256</v>
-      </c>
-      <c r="E35" s="40" t="s">
-        <v>127</v>
-      </c>
-      <c r="F35" s="39" t="s">
-        <v>128</v>
-      </c>
-      <c r="G35" s="40" t="s">
-        <v>129</v>
-      </c>
-      <c r="H35" s="41" t="s">
-        <v>130</v>
-      </c>
-      <c r="I35" s="36" t="s">
-        <v>53</v>
-      </c>
-      <c r="J35" s="36"/>
-      <c r="K35" s="57">
-        <v>1</v>
-      </c>
-      <c r="L35" s="40">
-        <f t="shared" ref="L35:L37" si="10">K35*5</f>
-        <v>5</v>
-      </c>
-      <c r="M35" s="73" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="36" spans="1:13" ht="48.75" thickBot="1">
+      <c r="M35" s="64" t="s">
+        <v>249</v>
+      </c>
+      <c r="O35" s="87"/>
+    </row>
+    <row r="36" spans="1:15" ht="48.75" thickBot="1">
       <c r="A36" s="2"/>
       <c r="B36" s="34">
         <f t="shared" si="0"/>
@@ -3131,8 +3194,8 @@
       <c r="C36" s="35" t="s">
         <v>121</v>
       </c>
-      <c r="D36" s="77" t="s">
-        <v>257</v>
+      <c r="D36" s="69" t="s">
+        <v>255</v>
       </c>
       <c r="E36" s="40" t="s">
         <v>127</v>
@@ -3146,39 +3209,44 @@
       <c r="H36" s="41" t="s">
         <v>130</v>
       </c>
-      <c r="I36" s="36"/>
+      <c r="I36" s="36" t="s">
+        <v>53</v>
+      </c>
       <c r="J36" s="36"/>
-      <c r="K36" s="56">
+      <c r="K36" s="57">
         <v>1</v>
       </c>
-      <c r="L36" s="37">
-        <f t="shared" si="10"/>
+      <c r="L36" s="40">
+        <f t="shared" ref="L36:L38" si="10">K36*5</f>
         <v>5</v>
       </c>
-      <c r="M36" s="36"/>
-    </row>
-    <row r="37" spans="1:13" ht="15.75" thickBot="1">
+      <c r="M36" s="64" t="s">
+        <v>249</v>
+      </c>
+      <c r="O36" s="87"/>
+    </row>
+    <row r="37" spans="1:15" ht="48.75" thickBot="1">
       <c r="A37" s="2"/>
       <c r="B37" s="34">
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
-      <c r="C37" s="43" t="s">
+      <c r="C37" s="35" t="s">
         <v>121</v>
       </c>
-      <c r="D37" s="72" t="s">
-        <v>131</v>
-      </c>
-      <c r="E37" s="37" t="s">
-        <v>132</v>
-      </c>
-      <c r="F37" s="36" t="s">
-        <v>133</v>
-      </c>
-      <c r="G37" s="37" t="s">
-        <v>134</v>
-      </c>
-      <c r="H37" s="38" t="s">
+      <c r="D37" s="68" t="s">
+        <v>256</v>
+      </c>
+      <c r="E37" s="40" t="s">
+        <v>127</v>
+      </c>
+      <c r="F37" s="39" t="s">
+        <v>128</v>
+      </c>
+      <c r="G37" s="40" t="s">
+        <v>129</v>
+      </c>
+      <c r="H37" s="41" t="s">
         <v>130</v>
       </c>
       <c r="I37" s="36" t="s">
@@ -3193,123 +3261,125 @@
         <v>5</v>
       </c>
       <c r="M37" s="36"/>
-    </row>
-    <row r="38" spans="1:13">
+      <c r="O37" s="87"/>
+    </row>
+    <row r="38" spans="1:15" ht="15.75" thickBot="1">
       <c r="A38" s="2"/>
       <c r="B38" s="34">
         <f t="shared" si="0"/>
         <v>29</v>
       </c>
-      <c r="C38" s="35" t="s">
-        <v>135</v>
-      </c>
-      <c r="D38" s="82" t="s">
-        <v>136</v>
-      </c>
-      <c r="E38" s="40" t="s">
-        <v>137</v>
-      </c>
-      <c r="F38" s="39" t="s">
-        <v>138</v>
-      </c>
-      <c r="G38" s="40" t="s">
-        <v>139</v>
-      </c>
-      <c r="H38" s="41" t="s">
-        <v>21</v>
-      </c>
-      <c r="I38" s="39" t="s">
-        <v>140</v>
-      </c>
-      <c r="J38" s="39"/>
-      <c r="K38" s="57">
-        <v>2</v>
-      </c>
-      <c r="L38" s="40">
-        <f t="shared" ref="L38:L39" si="11">K38*5</f>
-        <v>10</v>
-      </c>
-      <c r="M38" s="39"/>
-    </row>
-    <row r="39" spans="1:13">
+      <c r="C38" s="43" t="s">
+        <v>121</v>
+      </c>
+      <c r="D38" s="63" t="s">
+        <v>131</v>
+      </c>
+      <c r="E38" s="37" t="s">
+        <v>132</v>
+      </c>
+      <c r="F38" s="36" t="s">
+        <v>133</v>
+      </c>
+      <c r="G38" s="37" t="s">
+        <v>134</v>
+      </c>
+      <c r="H38" s="38" t="s">
+        <v>130</v>
+      </c>
+      <c r="I38" s="36" t="s">
+        <v>53</v>
+      </c>
+      <c r="J38" s="36"/>
+      <c r="K38" s="56">
+        <v>1</v>
+      </c>
+      <c r="L38" s="37">
+        <f t="shared" si="10"/>
+        <v>5</v>
+      </c>
+      <c r="M38" s="36"/>
+      <c r="O38" s="87"/>
+    </row>
+    <row r="39" spans="1:15">
       <c r="A39" s="2"/>
       <c r="B39" s="34">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="C39" s="43" t="s">
+      <c r="C39" s="35" t="s">
         <v>135</v>
       </c>
-      <c r="D39" s="72" t="s">
+      <c r="D39" s="73" t="s">
+        <v>136</v>
+      </c>
+      <c r="E39" s="40" t="s">
+        <v>137</v>
+      </c>
+      <c r="F39" s="39" t="s">
+        <v>138</v>
+      </c>
+      <c r="G39" s="40" t="s">
+        <v>139</v>
+      </c>
+      <c r="H39" s="41" t="s">
+        <v>21</v>
+      </c>
+      <c r="I39" s="39" t="s">
+        <v>140</v>
+      </c>
+      <c r="J39" s="39"/>
+      <c r="K39" s="57">
+        <v>2</v>
+      </c>
+      <c r="L39" s="40">
+        <f t="shared" ref="L39:L40" si="11">K39*5</f>
+        <v>10</v>
+      </c>
+      <c r="M39" s="39"/>
+      <c r="O39" s="87"/>
+    </row>
+    <row r="40" spans="1:15">
+      <c r="A40" s="2"/>
+      <c r="B40" s="34">
+        <f t="shared" si="0"/>
+        <v>31</v>
+      </c>
+      <c r="C40" s="43" t="s">
+        <v>135</v>
+      </c>
+      <c r="D40" s="63" t="s">
         <v>141</v>
       </c>
-      <c r="E39" s="37" t="s">
+      <c r="E40" s="37" t="s">
         <v>142</v>
       </c>
-      <c r="F39" s="36" t="s">
+      <c r="F40" s="36" t="s">
         <v>138</v>
       </c>
-      <c r="G39" s="37" t="s">
+      <c r="G40" s="37" t="s">
         <v>143</v>
       </c>
-      <c r="H39" s="38" t="s">
+      <c r="H40" s="38" t="s">
         <v>21</v>
       </c>
-      <c r="I39" s="36" t="s">
+      <c r="I40" s="36" t="s">
         <v>144</v>
       </c>
-      <c r="J39" s="36"/>
-      <c r="K39" s="56">
+      <c r="J40" s="36"/>
+      <c r="K40" s="56">
         <v>1</v>
       </c>
-      <c r="L39" s="37">
+      <c r="L40" s="37">
         <f t="shared" si="11"/>
         <v>5</v>
       </c>
-      <c r="M39" s="73" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="40" spans="1:13" ht="24.75" thickBot="1">
-      <c r="A40" s="2"/>
-      <c r="B40" s="34">
-        <f t="shared" si="0"/>
-        <v>31</v>
-      </c>
-      <c r="C40" s="35" t="s">
-        <v>135</v>
-      </c>
-      <c r="D40" s="82" t="s">
-        <v>145</v>
-      </c>
-      <c r="E40" s="40" t="s">
-        <v>146</v>
-      </c>
-      <c r="F40" s="39" t="s">
-        <v>138</v>
-      </c>
-      <c r="G40" s="81" t="s">
-        <v>147</v>
-      </c>
-      <c r="H40" s="41" t="s">
-        <v>148</v>
-      </c>
-      <c r="I40" s="39" t="s">
-        <v>149</v>
-      </c>
-      <c r="J40" s="39"/>
-      <c r="K40" s="57">
-        <v>1</v>
-      </c>
-      <c r="L40" s="40">
-        <f t="shared" ref="L40:L48" si="12">K40*5</f>
-        <v>5</v>
-      </c>
-      <c r="M40" s="73" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="41" spans="1:13" ht="15.75" thickBot="1">
+      <c r="M40" s="64" t="s">
+        <v>249</v>
+      </c>
+      <c r="O40" s="87"/>
+    </row>
+    <row r="41" spans="1:15" ht="24.75" thickBot="1">
       <c r="A41" s="2"/>
       <c r="B41" s="34">
         <f t="shared" si="0"/>
@@ -3318,115 +3388,118 @@
       <c r="C41" s="35" t="s">
         <v>135</v>
       </c>
-      <c r="D41" s="82" t="s">
-        <v>258</v>
-      </c>
-      <c r="E41" s="81" t="s">
+      <c r="D41" s="73" t="s">
+        <v>145</v>
+      </c>
+      <c r="E41" s="40" t="s">
+        <v>146</v>
+      </c>
+      <c r="F41" s="39" t="s">
+        <v>138</v>
+      </c>
+      <c r="G41" s="72" t="s">
+        <v>147</v>
+      </c>
+      <c r="H41" s="41" t="s">
+        <v>148</v>
+      </c>
+      <c r="I41" s="39" t="s">
+        <v>149</v>
+      </c>
+      <c r="J41" s="39"/>
+      <c r="K41" s="57">
+        <v>1</v>
+      </c>
+      <c r="L41" s="40">
+        <f t="shared" ref="L41:L49" si="12">K41*5</f>
+        <v>5</v>
+      </c>
+      <c r="M41" s="64" t="s">
+        <v>249</v>
+      </c>
+      <c r="O41" s="87"/>
+    </row>
+    <row r="42" spans="1:15" ht="15.75" thickBot="1">
+      <c r="A42" s="2"/>
+      <c r="B42" s="34">
+        <f t="shared" si="0"/>
+        <v>33</v>
+      </c>
+      <c r="C42" s="35" t="s">
+        <v>135</v>
+      </c>
+      <c r="D42" s="73" t="s">
+        <v>257</v>
+      </c>
+      <c r="E42" s="72" t="s">
         <v>150</v>
       </c>
-      <c r="F41" s="76" t="s">
+      <c r="F42" s="67" t="s">
         <v>138</v>
       </c>
-      <c r="G41" s="81" t="s">
+      <c r="G42" s="72" t="s">
         <v>151</v>
       </c>
-      <c r="H41" s="38" t="s">
+      <c r="H42" s="38" t="s">
         <v>21</v>
       </c>
-      <c r="I41" s="39" t="s">
+      <c r="I42" s="39" t="s">
         <v>152</v>
       </c>
-      <c r="J41" s="36"/>
-      <c r="K41" s="56">
+      <c r="J42" s="36"/>
+      <c r="K42" s="56">
         <v>1</v>
       </c>
-      <c r="L41" s="37">
+      <c r="L42" s="37">
         <f t="shared" si="12"/>
         <v>5</v>
       </c>
-      <c r="M41" s="73" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="42" spans="1:13" ht="24.75" thickBot="1">
-      <c r="A42" s="2"/>
-      <c r="B42" s="34">
-        <f t="shared" si="0"/>
-        <v>33</v>
-      </c>
-      <c r="C42" s="35" t="s">
-        <v>135</v>
-      </c>
-      <c r="D42" s="82" t="s">
-        <v>153</v>
-      </c>
-      <c r="E42" s="40" t="s">
-        <v>154</v>
-      </c>
-      <c r="F42" s="39" t="s">
-        <v>155</v>
-      </c>
-      <c r="G42" s="40" t="s">
-        <v>156</v>
-      </c>
-      <c r="H42" s="41" t="s">
-        <v>157</v>
-      </c>
-      <c r="I42" s="39" t="s">
-        <v>158</v>
-      </c>
-      <c r="J42" s="39"/>
-      <c r="K42" s="57">
-        <v>1</v>
-      </c>
-      <c r="L42" s="40">
-        <f>K42*5</f>
-        <v>5</v>
-      </c>
-      <c r="M42" s="73" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="43" spans="1:13" ht="15.75" thickBot="1">
+      <c r="M42" s="64" t="s">
+        <v>249</v>
+      </c>
+      <c r="O42" s="87"/>
+    </row>
+    <row r="43" spans="1:15" ht="24.75" thickBot="1">
       <c r="A43" s="2"/>
       <c r="B43" s="34">
         <f t="shared" si="0"/>
         <v>34</v>
       </c>
-      <c r="C43" s="43" t="s">
+      <c r="C43" s="35" t="s">
         <v>135</v>
       </c>
-      <c r="D43" s="77" t="s">
-        <v>260</v>
-      </c>
-      <c r="E43" s="37" t="s">
-        <v>159</v>
-      </c>
-      <c r="F43" s="36" t="s">
-        <v>138</v>
-      </c>
-      <c r="G43" s="37" t="s">
-        <v>160</v>
-      </c>
-      <c r="H43" s="38" t="s">
-        <v>21</v>
-      </c>
-      <c r="I43" s="36" t="s">
-        <v>161</v>
-      </c>
-      <c r="J43" s="36"/>
-      <c r="K43" s="56">
+      <c r="D43" s="73" t="s">
+        <v>153</v>
+      </c>
+      <c r="E43" s="40" t="s">
+        <v>154</v>
+      </c>
+      <c r="F43" s="39" t="s">
+        <v>155</v>
+      </c>
+      <c r="G43" s="40" t="s">
+        <v>156</v>
+      </c>
+      <c r="H43" s="41" t="s">
+        <v>157</v>
+      </c>
+      <c r="I43" s="39" t="s">
+        <v>158</v>
+      </c>
+      <c r="J43" s="39"/>
+      <c r="K43" s="57">
         <v>1</v>
       </c>
-      <c r="L43" s="37">
-        <f t="shared" ref="L43" si="13">K43*5</f>
+      <c r="L43" s="40">
+        <f>K43*5</f>
         <v>5</v>
       </c>
-      <c r="M43" s="73" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="44" spans="1:13" ht="15.75" thickBot="1">
+      <c r="M43" s="64" t="s">
+        <v>249</v>
+      </c>
+      <c r="O43" s="87"/>
+    </row>
+    <row r="44" spans="1:15" ht="15.75" thickBot="1">
       <c r="A44" s="2"/>
       <c r="B44" s="34">
         <f t="shared" si="0"/>
@@ -3435,37 +3508,38 @@
       <c r="C44" s="43" t="s">
         <v>135</v>
       </c>
-      <c r="D44" s="77" t="s">
-        <v>261</v>
-      </c>
-      <c r="E44" s="40" t="s">
-        <v>162</v>
-      </c>
-      <c r="F44" s="39" t="s">
+      <c r="D44" s="68" t="s">
+        <v>259</v>
+      </c>
+      <c r="E44" s="37" t="s">
+        <v>159</v>
+      </c>
+      <c r="F44" s="36" t="s">
         <v>138</v>
       </c>
-      <c r="G44" s="81" t="s">
-        <v>163</v>
-      </c>
-      <c r="H44" s="41" t="s">
+      <c r="G44" s="37" t="s">
+        <v>160</v>
+      </c>
+      <c r="H44" s="38" t="s">
         <v>21</v>
       </c>
-      <c r="I44" s="39" t="s">
-        <v>164</v>
-      </c>
-      <c r="J44" s="39"/>
-      <c r="K44" s="57">
-        <v>2</v>
-      </c>
-      <c r="L44" s="40">
-        <f>K44*5</f>
-        <v>10</v>
-      </c>
-      <c r="M44" s="73" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="45" spans="1:13" ht="15.75" thickBot="1">
+      <c r="I44" s="36" t="s">
+        <v>161</v>
+      </c>
+      <c r="J44" s="36"/>
+      <c r="K44" s="56">
+        <v>1</v>
+      </c>
+      <c r="L44" s="37">
+        <f t="shared" ref="L44" si="13">K44*5</f>
+        <v>5</v>
+      </c>
+      <c r="M44" s="64" t="s">
+        <v>249</v>
+      </c>
+      <c r="O44" s="87"/>
+    </row>
+    <row r="45" spans="1:15" ht="15.75" thickBot="1">
       <c r="A45" s="2"/>
       <c r="B45" s="34">
         <f t="shared" si="0"/>
@@ -3474,35 +3548,38 @@
       <c r="C45" s="43" t="s">
         <v>135</v>
       </c>
-      <c r="D45" s="77" t="s">
-        <v>262</v>
-      </c>
-      <c r="E45" s="37" t="s">
-        <v>165</v>
-      </c>
-      <c r="F45" s="36" t="s">
+      <c r="D45" s="68" t="s">
+        <v>260</v>
+      </c>
+      <c r="E45" s="40" t="s">
+        <v>162</v>
+      </c>
+      <c r="F45" s="39" t="s">
         <v>138</v>
       </c>
-      <c r="G45" s="37" t="s">
-        <v>166</v>
-      </c>
-      <c r="H45" s="38" t="s">
+      <c r="G45" s="72" t="s">
+        <v>163</v>
+      </c>
+      <c r="H45" s="41" t="s">
         <v>21</v>
       </c>
-      <c r="I45" s="36" t="s">
-        <v>167</v>
-      </c>
-      <c r="J45" s="36"/>
-      <c r="K45" s="56">
+      <c r="I45" s="39" t="s">
+        <v>164</v>
+      </c>
+      <c r="J45" s="39"/>
+      <c r="K45" s="57">
         <v>2</v>
       </c>
-      <c r="L45" s="37">
+      <c r="L45" s="40">
         <f>K45*5</f>
         <v>10</v>
       </c>
-      <c r="M45" s="36"/>
-    </row>
-    <row r="46" spans="1:13" ht="15.75" thickBot="1">
+      <c r="M45" s="64" t="s">
+        <v>249</v>
+      </c>
+      <c r="O45" s="87"/>
+    </row>
+    <row r="46" spans="1:15" ht="15.75" thickBot="1">
       <c r="A46" s="2"/>
       <c r="B46" s="34">
         <f t="shared" si="0"/>
@@ -3511,35 +3588,36 @@
       <c r="C46" s="43" t="s">
         <v>135</v>
       </c>
-      <c r="D46" s="77" t="s">
-        <v>263</v>
-      </c>
-      <c r="E46" s="81" t="s">
-        <v>162</v>
-      </c>
-      <c r="F46" s="75" t="s">
+      <c r="D46" s="68" t="s">
+        <v>261</v>
+      </c>
+      <c r="E46" s="37" t="s">
+        <v>165</v>
+      </c>
+      <c r="F46" s="36" t="s">
         <v>138</v>
       </c>
-      <c r="G46" s="81" t="s">
-        <v>163</v>
+      <c r="G46" s="37" t="s">
+        <v>166</v>
       </c>
       <c r="H46" s="38" t="s">
         <v>21</v>
       </c>
-      <c r="I46" s="39" t="s">
-        <v>164</v>
+      <c r="I46" s="36" t="s">
+        <v>167</v>
       </c>
       <c r="J46" s="36"/>
       <c r="K46" s="56">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L46" s="37">
         <f>K46*5</f>
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="M46" s="36"/>
-    </row>
-    <row r="47" spans="1:13" ht="15.75" thickBot="1">
+      <c r="O46" s="87"/>
+    </row>
+    <row r="47" spans="1:15" ht="15.75" thickBot="1">
       <c r="A47" s="2"/>
       <c r="B47" s="34">
         <f t="shared" si="0"/>
@@ -3548,35 +3626,36 @@
       <c r="C47" s="43" t="s">
         <v>135</v>
       </c>
-      <c r="D47" s="77" t="s">
-        <v>266</v>
-      </c>
-      <c r="E47" s="81" t="s">
-        <v>265</v>
-      </c>
-      <c r="F47" s="75" t="s">
+      <c r="D47" s="68" t="s">
+        <v>262</v>
+      </c>
+      <c r="E47" s="72" t="s">
+        <v>162</v>
+      </c>
+      <c r="F47" s="66" t="s">
         <v>138</v>
       </c>
-      <c r="G47" s="81" t="s">
-        <v>264</v>
+      <c r="G47" s="72" t="s">
+        <v>163</v>
       </c>
       <c r="H47" s="38" t="s">
         <v>21</v>
       </c>
       <c r="I47" s="39" t="s">
-        <v>177</v>
+        <v>164</v>
       </c>
       <c r="J47" s="36"/>
       <c r="K47" s="56">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L47" s="37">
         <f>K47*5</f>
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="M47" s="36"/>
-    </row>
-    <row r="48" spans="1:13" ht="15.75" thickBot="1">
+      <c r="O47" s="87"/>
+    </row>
+    <row r="48" spans="1:15" ht="15.75" thickBot="1">
       <c r="A48" s="2"/>
       <c r="B48" s="34">
         <f t="shared" si="0"/>
@@ -3585,372 +3664,383 @@
       <c r="C48" s="43" t="s">
         <v>135</v>
       </c>
-      <c r="D48" s="77" t="s">
-        <v>259</v>
-      </c>
-      <c r="E48" s="37" t="s">
-        <v>150</v>
-      </c>
-      <c r="F48" s="36" t="s">
+      <c r="D48" s="68" t="s">
+        <v>265</v>
+      </c>
+      <c r="E48" s="72" t="s">
+        <v>264</v>
+      </c>
+      <c r="F48" s="66" t="s">
         <v>138</v>
       </c>
-      <c r="G48" s="37" t="s">
-        <v>151</v>
+      <c r="G48" s="72" t="s">
+        <v>263</v>
       </c>
       <c r="H48" s="38" t="s">
         <v>21</v>
       </c>
-      <c r="I48" s="36" t="s">
-        <v>152</v>
+      <c r="I48" s="39" t="s">
+        <v>177</v>
       </c>
       <c r="J48" s="36"/>
       <c r="K48" s="56">
+        <v>2</v>
+      </c>
+      <c r="L48" s="37">
+        <f>K48*5</f>
+        <v>10</v>
+      </c>
+      <c r="M48" s="36"/>
+      <c r="O48" s="87"/>
+    </row>
+    <row r="49" spans="1:15" ht="15.75" thickBot="1">
+      <c r="A49" s="2"/>
+      <c r="B49" s="34">
+        <f t="shared" si="0"/>
+        <v>40</v>
+      </c>
+      <c r="C49" s="43" t="s">
+        <v>135</v>
+      </c>
+      <c r="D49" s="68" t="s">
+        <v>258</v>
+      </c>
+      <c r="E49" s="37" t="s">
+        <v>150</v>
+      </c>
+      <c r="F49" s="36" t="s">
+        <v>138</v>
+      </c>
+      <c r="G49" s="37" t="s">
+        <v>151</v>
+      </c>
+      <c r="H49" s="38" t="s">
+        <v>21</v>
+      </c>
+      <c r="I49" s="36" t="s">
+        <v>152</v>
+      </c>
+      <c r="J49" s="36"/>
+      <c r="K49" s="56">
         <v>5</v>
       </c>
-      <c r="L48" s="37">
+      <c r="L49" s="37">
         <f t="shared" si="12"/>
         <v>25</v>
       </c>
-      <c r="M48" s="75"/>
-    </row>
-    <row r="49" spans="1:13" ht="15.75" thickBot="1">
-      <c r="A49" s="2"/>
-      <c r="B49" s="34">
-        <f t="shared" si="0"/>
-        <v>40</v>
-      </c>
-      <c r="C49" s="43" t="s">
-        <v>135</v>
-      </c>
-      <c r="D49" s="77" t="s">
-        <v>168</v>
-      </c>
-      <c r="E49" s="37" t="s">
-        <v>169</v>
-      </c>
-      <c r="F49" s="36" t="s">
-        <v>155</v>
-      </c>
-      <c r="G49" s="37" t="s">
-        <v>170</v>
-      </c>
-      <c r="H49" s="38" t="s">
-        <v>21</v>
-      </c>
-      <c r="I49" s="36" t="s">
-        <v>152</v>
-      </c>
-      <c r="J49" s="36"/>
-      <c r="K49" s="56">
-        <v>2</v>
-      </c>
-      <c r="L49" s="37">
-        <f>K49*5</f>
-        <v>10</v>
-      </c>
-      <c r="M49" s="36"/>
-    </row>
-    <row r="50" spans="1:13">
+      <c r="M49" s="66"/>
+      <c r="O49" s="87"/>
+    </row>
+    <row r="50" spans="1:15" ht="15.75" thickBot="1">
       <c r="A50" s="2"/>
       <c r="B50" s="34">
         <f t="shared" si="0"/>
         <v>41</v>
       </c>
-      <c r="C50" s="35" t="s">
+      <c r="C50" s="43" t="s">
         <v>135</v>
       </c>
-      <c r="D50" s="77" t="s">
-        <v>267</v>
-      </c>
-      <c r="E50" s="40" t="s">
-        <v>171</v>
-      </c>
-      <c r="F50" s="39" t="s">
-        <v>138</v>
-      </c>
-      <c r="G50" s="40" t="s">
-        <v>172</v>
-      </c>
-      <c r="H50" s="41" t="s">
+      <c r="D50" s="68" t="s">
+        <v>168</v>
+      </c>
+      <c r="E50" s="37" t="s">
+        <v>169</v>
+      </c>
+      <c r="F50" s="36" t="s">
+        <v>155</v>
+      </c>
+      <c r="G50" s="37" t="s">
+        <v>170</v>
+      </c>
+      <c r="H50" s="38" t="s">
         <v>21</v>
       </c>
-      <c r="I50" s="39" t="s">
-        <v>173</v>
-      </c>
-      <c r="J50" s="39"/>
-      <c r="K50" s="57">
-        <v>1</v>
-      </c>
-      <c r="L50" s="40">
-        <f t="shared" ref="L50:L53" si="14">K50*5</f>
-        <v>5</v>
-      </c>
-      <c r="M50" s="39"/>
-    </row>
-    <row r="51" spans="1:13" ht="15.75" thickBot="1">
+      <c r="I50" s="36" t="s">
+        <v>152</v>
+      </c>
+      <c r="J50" s="36"/>
+      <c r="K50" s="56">
+        <v>2</v>
+      </c>
+      <c r="L50" s="37">
+        <f>K50*5</f>
+        <v>10</v>
+      </c>
+      <c r="M50" s="36"/>
+      <c r="O50" s="87"/>
+    </row>
+    <row r="51" spans="1:15" ht="15.75" thickBot="1">
       <c r="A51" s="2"/>
       <c r="B51" s="34">
         <f t="shared" si="0"/>
         <v>42</v>
       </c>
-      <c r="C51" s="43" t="s">
+      <c r="C51" s="35" t="s">
         <v>135</v>
       </c>
-      <c r="D51" s="77" t="s">
+      <c r="D51" s="68" t="s">
+        <v>266</v>
+      </c>
+      <c r="E51" s="40" t="s">
+        <v>171</v>
+      </c>
+      <c r="F51" s="39" t="s">
+        <v>138</v>
+      </c>
+      <c r="G51" s="40" t="s">
+        <v>172</v>
+      </c>
+      <c r="H51" s="41" t="s">
+        <v>21</v>
+      </c>
+      <c r="I51" s="39" t="s">
+        <v>173</v>
+      </c>
+      <c r="J51" s="39"/>
+      <c r="K51" s="57">
+        <v>1</v>
+      </c>
+      <c r="L51" s="40">
+        <f t="shared" ref="L51:L55" si="14">K51*5</f>
+        <v>5</v>
+      </c>
+      <c r="M51" s="39"/>
+      <c r="O51" s="87"/>
+    </row>
+    <row r="52" spans="1:15" ht="15.75" thickBot="1">
+      <c r="A52" s="2"/>
+      <c r="B52" s="34">
+        <v>43</v>
+      </c>
+      <c r="C52" s="35" t="s">
+        <v>135</v>
+      </c>
+      <c r="D52" s="68" t="s">
+        <v>274</v>
+      </c>
+      <c r="E52" s="37" t="s">
+        <v>175</v>
+      </c>
+      <c r="F52" s="39" t="s">
+        <v>138</v>
+      </c>
+      <c r="G52" s="37" t="s">
+        <v>176</v>
+      </c>
+      <c r="H52" s="41" t="s">
+        <v>21</v>
+      </c>
+      <c r="I52" s="36" t="s">
+        <v>177</v>
+      </c>
+      <c r="J52" s="36"/>
+      <c r="K52" s="56">
+        <v>6</v>
+      </c>
+      <c r="L52" s="37">
+        <f t="shared" si="14"/>
+        <v>30</v>
+      </c>
+      <c r="M52" s="64" t="s">
+        <v>249</v>
+      </c>
+      <c r="O52" s="87"/>
+    </row>
+    <row r="53" spans="1:15" ht="15.75" thickBot="1">
+      <c r="A53" s="2"/>
+      <c r="B53" s="34">
+        <f t="shared" si="0"/>
+        <v>44</v>
+      </c>
+      <c r="C53" s="43" t="s">
+        <v>135</v>
+      </c>
+      <c r="D53" s="68" t="s">
         <v>174</v>
       </c>
-      <c r="E51" s="37" t="s">
+      <c r="E53" s="37" t="s">
         <v>175</v>
       </c>
-      <c r="F51" s="75" t="s">
+      <c r="F53" s="66" t="s">
         <v>138</v>
       </c>
-      <c r="G51" s="37" t="s">
+      <c r="G53" s="37" t="s">
         <v>176</v>
       </c>
-      <c r="H51" s="38" t="s">
+      <c r="H53" s="38" t="s">
         <v>21</v>
       </c>
-      <c r="I51" s="36" t="s">
+      <c r="I53" s="36" t="s">
         <v>177</v>
       </c>
-      <c r="J51" s="36"/>
-      <c r="K51" s="56">
+      <c r="J53" s="36"/>
+      <c r="K53" s="56">
         <v>4</v>
       </c>
-      <c r="L51" s="37">
+      <c r="L53" s="37">
         <f t="shared" si="14"/>
         <v>20</v>
       </c>
-      <c r="M51" s="36"/>
-    </row>
-    <row r="52" spans="1:13" ht="15.75" thickBot="1">
-      <c r="A52" s="2"/>
-      <c r="B52" s="34">
-        <f t="shared" si="0"/>
-        <v>43</v>
-      </c>
-      <c r="C52" s="43" t="s">
+      <c r="M53" s="36"/>
+      <c r="O53" s="87"/>
+    </row>
+    <row r="54" spans="1:15" ht="15.75" thickBot="1">
+      <c r="A54" s="2"/>
+      <c r="B54" s="34">
+        <f t="shared" si="0"/>
+        <v>45</v>
+      </c>
+      <c r="C54" s="43" t="s">
         <v>135</v>
       </c>
-      <c r="D52" s="77" t="s">
-        <v>268</v>
-      </c>
-      <c r="E52" s="81" t="s">
+      <c r="D54" s="68" t="s">
+        <v>267</v>
+      </c>
+      <c r="E54" s="72" t="s">
         <v>171</v>
       </c>
-      <c r="F52" s="75" t="s">
+      <c r="F54" s="66" t="s">
         <v>138</v>
       </c>
-      <c r="G52" s="81" t="s">
+      <c r="G54" s="72" t="s">
         <v>172</v>
       </c>
-      <c r="H52" s="38" t="s">
+      <c r="H54" s="38" t="s">
         <v>21</v>
       </c>
-      <c r="I52" s="39" t="s">
+      <c r="I54" s="39" t="s">
         <v>173</v>
       </c>
-      <c r="J52" s="36"/>
-      <c r="K52" s="56">
+      <c r="J54" s="36"/>
+      <c r="K54" s="56">
         <v>1</v>
       </c>
-      <c r="L52" s="37">
+      <c r="L54" s="37">
         <f t="shared" si="14"/>
         <v>5</v>
       </c>
-      <c r="M52" s="73" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="53" spans="1:13" ht="15.75" thickBot="1">
-      <c r="A53" s="2"/>
-      <c r="B53" s="34">
-        <f t="shared" si="0"/>
-        <v>44</v>
-      </c>
-      <c r="C53" s="43" t="s">
+      <c r="M54" s="64" t="s">
+        <v>249</v>
+      </c>
+      <c r="O54" s="87"/>
+    </row>
+    <row r="55" spans="1:15" ht="15.75" thickBot="1">
+      <c r="A55" s="2"/>
+      <c r="B55" s="34">
+        <f t="shared" si="0"/>
+        <v>46</v>
+      </c>
+      <c r="C55" s="43" t="s">
         <v>135</v>
       </c>
-      <c r="D53" s="77" t="s">
-        <v>269</v>
-      </c>
-      <c r="E53" s="81" t="s">
+      <c r="D55" s="68" t="s">
+        <v>268</v>
+      </c>
+      <c r="E55" s="72" t="s">
         <v>165</v>
       </c>
-      <c r="F53" s="75" t="s">
+      <c r="F55" s="66" t="s">
         <v>138</v>
       </c>
-      <c r="G53" s="81" t="s">
+      <c r="G55" s="72" t="s">
         <v>166</v>
       </c>
-      <c r="H53" s="38" t="s">
+      <c r="H55" s="38" t="s">
         <v>21</v>
       </c>
-      <c r="I53" s="36" t="s">
+      <c r="I55" s="36" t="s">
         <v>167</v>
       </c>
-      <c r="J53" s="36"/>
-      <c r="K53" s="56">
+      <c r="J55" s="36"/>
+      <c r="K55" s="56">
         <v>1</v>
       </c>
-      <c r="L53" s="37">
+      <c r="L55" s="37">
         <f t="shared" si="14"/>
         <v>5</v>
       </c>
-      <c r="M53" s="73" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="54" spans="1:13" ht="15.75" thickBot="1">
-      <c r="A54" s="2"/>
-      <c r="B54" s="34">
-        <f t="shared" si="0"/>
-        <v>45</v>
-      </c>
-      <c r="C54" s="43" t="s">
+      <c r="M55" s="64" t="s">
+        <v>249</v>
+      </c>
+      <c r="O55" s="87"/>
+    </row>
+    <row r="56" spans="1:15" ht="15.75" thickBot="1">
+      <c r="A56" s="2"/>
+      <c r="B56" s="34">
+        <f t="shared" si="0"/>
+        <v>47</v>
+      </c>
+      <c r="C56" s="43" t="s">
         <v>135</v>
       </c>
-      <c r="D54" s="77" t="s">
+      <c r="D56" s="68" t="s">
         <v>178</v>
       </c>
-      <c r="E54" s="40" t="s">
+      <c r="E56" s="40" t="s">
         <v>179</v>
       </c>
-      <c r="F54" s="39" t="s">
+      <c r="F56" s="39" t="s">
         <v>138</v>
       </c>
-      <c r="G54" s="40" t="s">
+      <c r="G56" s="40" t="s">
         <v>180</v>
       </c>
-      <c r="H54" s="41" t="s">
+      <c r="H56" s="41" t="s">
         <v>21</v>
       </c>
-      <c r="I54" s="39" t="s">
+      <c r="I56" s="39" t="s">
         <v>181</v>
       </c>
-      <c r="J54" s="39"/>
-      <c r="K54" s="57">
+      <c r="J56" s="39"/>
+      <c r="K56" s="57">
         <v>2</v>
       </c>
-      <c r="L54" s="40">
-        <f t="shared" ref="L54:L56" si="15">K54*5</f>
+      <c r="L56" s="40">
+        <f t="shared" ref="L56:L58" si="15">K56*5</f>
         <v>10</v>
       </c>
-      <c r="M54" s="39"/>
-    </row>
-    <row r="55" spans="1:13" ht="15.75" thickBot="1">
-      <c r="A55" s="2"/>
-      <c r="B55" s="34">
-        <f t="shared" si="0"/>
-        <v>46</v>
-      </c>
-      <c r="C55" s="43" t="s">
+      <c r="M56" s="39"/>
+      <c r="O56" s="87"/>
+    </row>
+    <row r="57" spans="1:15" ht="15.75" thickBot="1">
+      <c r="A57" s="2"/>
+      <c r="B57" s="34">
+        <f t="shared" si="0"/>
+        <v>48</v>
+      </c>
+      <c r="C57" s="43" t="s">
         <v>135</v>
       </c>
-      <c r="D55" s="77" t="s">
-        <v>270</v>
-      </c>
-      <c r="E55" s="81" t="s">
+      <c r="D57" s="68" t="s">
+        <v>269</v>
+      </c>
+      <c r="E57" s="72" t="s">
         <v>159</v>
       </c>
-      <c r="F55" s="76" t="s">
+      <c r="F57" s="67" t="s">
         <v>138</v>
       </c>
-      <c r="G55" s="37" t="s">
+      <c r="G57" s="37" t="s">
         <v>160</v>
       </c>
-      <c r="H55" s="41" t="s">
+      <c r="H57" s="41" t="s">
         <v>21</v>
       </c>
-      <c r="I55" s="39" t="s">
+      <c r="I57" s="39" t="s">
         <v>161</v>
       </c>
-      <c r="J55" s="36"/>
-      <c r="K55" s="56">
+      <c r="J57" s="36"/>
+      <c r="K57" s="56">
         <v>2</v>
       </c>
-      <c r="L55" s="37">
+      <c r="L57" s="37">
         <f t="shared" si="15"/>
         <v>10</v>
       </c>
-      <c r="M55" s="36"/>
-    </row>
-    <row r="56" spans="1:13" ht="48.75" thickBot="1">
-      <c r="A56" s="2"/>
-      <c r="B56" s="34">
-        <f t="shared" si="0"/>
-        <v>47</v>
-      </c>
-      <c r="C56" s="43" t="s">
-        <v>182</v>
-      </c>
-      <c r="D56" s="72" t="s">
-        <v>183</v>
-      </c>
-      <c r="E56" s="37" t="s">
-        <v>184</v>
-      </c>
-      <c r="F56" s="36" t="s">
-        <v>185</v>
-      </c>
-      <c r="G56" s="37" t="s">
-        <v>185</v>
-      </c>
-      <c r="H56" s="38" t="s">
-        <v>186</v>
-      </c>
-      <c r="I56" s="36" t="s">
-        <v>53</v>
-      </c>
-      <c r="J56" s="36"/>
-      <c r="K56" s="56">
-        <v>1</v>
-      </c>
-      <c r="L56" s="37">
-        <f t="shared" si="15"/>
-        <v>5</v>
-      </c>
-      <c r="M56" s="36"/>
-    </row>
-    <row r="57" spans="1:13" ht="24">
-      <c r="A57" s="2"/>
-      <c r="B57" s="34">
-        <f t="shared" si="0"/>
-        <v>48</v>
-      </c>
-      <c r="C57" s="35" t="s">
-        <v>187</v>
-      </c>
-      <c r="D57" s="39" t="s">
-        <v>188</v>
-      </c>
-      <c r="E57" s="40" t="s">
-        <v>189</v>
-      </c>
-      <c r="F57" s="39" t="s">
-        <v>190</v>
-      </c>
-      <c r="G57" s="39" t="s">
-        <v>190</v>
-      </c>
-      <c r="H57" s="41" t="s">
-        <v>191</v>
-      </c>
-      <c r="I57" s="36" t="s">
-        <v>53</v>
-      </c>
-      <c r="J57" s="36"/>
-      <c r="K57" s="57">
-        <v>4</v>
-      </c>
-      <c r="L57" s="40">
-        <f t="shared" ref="L57:L58" si="16">K57*5</f>
-        <v>20</v>
-      </c>
-      <c r="M57" s="39"/>
-    </row>
-    <row r="58" spans="1:13" ht="48">
+      <c r="M57" s="36"/>
+      <c r="O57" s="87"/>
+    </row>
+    <row r="58" spans="1:15" ht="48.75" thickBot="1">
       <c r="A58" s="2"/>
       <c r="B58" s="34">
         <f t="shared" si="0"/>
@@ -3959,17 +4049,17 @@
       <c r="C58" s="43" t="s">
         <v>182</v>
       </c>
-      <c r="D58" s="36" t="s">
-        <v>192</v>
+      <c r="D58" s="63" t="s">
+        <v>183</v>
       </c>
       <c r="E58" s="37" t="s">
-        <v>193</v>
+        <v>184</v>
       </c>
       <c r="F58" s="36" t="s">
-        <v>194</v>
+        <v>185</v>
       </c>
       <c r="G58" s="37" t="s">
-        <v>195</v>
+        <v>185</v>
       </c>
       <c r="H58" s="38" t="s">
         <v>186</v>
@@ -3982,71 +4072,73 @@
         <v>1</v>
       </c>
       <c r="L58" s="37">
-        <f t="shared" si="16"/>
+        <f t="shared" si="15"/>
         <v>5</v>
       </c>
       <c r="M58" s="36"/>
-    </row>
-    <row r="59" spans="1:13" ht="24">
+      <c r="O58" s="87"/>
+    </row>
+    <row r="59" spans="1:15" ht="24">
       <c r="A59" s="2"/>
       <c r="B59" s="34">
         <f t="shared" si="0"/>
         <v>50</v>
       </c>
       <c r="C59" s="35" t="s">
-        <v>121</v>
+        <v>187</v>
       </c>
       <c r="D59" s="39" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
       <c r="E59" s="40" t="s">
-        <v>197</v>
+        <v>189</v>
       </c>
       <c r="F59" s="39" t="s">
-        <v>198</v>
-      </c>
-      <c r="G59" s="40" t="s">
-        <v>199</v>
+        <v>190</v>
+      </c>
+      <c r="G59" s="39" t="s">
+        <v>190</v>
       </c>
       <c r="H59" s="41" t="s">
-        <v>200</v>
+        <v>191</v>
       </c>
       <c r="I59" s="36" t="s">
         <v>53</v>
       </c>
       <c r="J59" s="36"/>
       <c r="K59" s="57">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L59" s="40">
-        <f t="shared" ref="L59:L60" si="17">K59*5</f>
-        <v>5</v>
+        <f t="shared" ref="L59:L60" si="16">K59*5</f>
+        <v>20</v>
       </c>
       <c r="M59" s="39"/>
-    </row>
-    <row r="60" spans="1:13" ht="24">
+      <c r="O59" s="87"/>
+    </row>
+    <row r="60" spans="1:15" ht="48">
       <c r="A60" s="2"/>
       <c r="B60" s="34">
         <f t="shared" si="0"/>
         <v>51</v>
       </c>
       <c r="C60" s="43" t="s">
-        <v>201</v>
+        <v>182</v>
       </c>
       <c r="D60" s="36" t="s">
-        <v>202</v>
+        <v>192</v>
       </c>
       <c r="E60" s="37" t="s">
-        <v>203</v>
+        <v>193</v>
       </c>
       <c r="F60" s="36" t="s">
-        <v>204</v>
+        <v>194</v>
       </c>
       <c r="G60" s="37" t="s">
-        <v>205</v>
+        <v>195</v>
       </c>
       <c r="H60" s="38" t="s">
-        <v>206</v>
+        <v>186</v>
       </c>
       <c r="I60" s="36" t="s">
         <v>53</v>
@@ -4056,36 +4148,35 @@
         <v>1</v>
       </c>
       <c r="L60" s="37">
-        <f t="shared" si="17"/>
+        <f t="shared" si="16"/>
         <v>5</v>
       </c>
-      <c r="M60" s="73" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="61" spans="1:13" ht="36">
+      <c r="M60" s="36"/>
+      <c r="O60" s="87"/>
+    </row>
+    <row r="61" spans="1:15" ht="24">
       <c r="A61" s="2"/>
       <c r="B61" s="34">
         <f t="shared" si="0"/>
         <v>52</v>
       </c>
       <c r="C61" s="35" t="s">
-        <v>201</v>
+        <v>121</v>
       </c>
       <c r="D61" s="39" t="s">
-        <v>207</v>
+        <v>196</v>
       </c>
       <c r="E61" s="40" t="s">
-        <v>208</v>
+        <v>197</v>
       </c>
       <c r="F61" s="39" t="s">
-        <v>209</v>
+        <v>198</v>
       </c>
       <c r="G61" s="40" t="s">
-        <v>210</v>
+        <v>199</v>
       </c>
       <c r="H61" s="41" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
       <c r="I61" s="36" t="s">
         <v>53</v>
@@ -4095,36 +4186,35 @@
         <v>1</v>
       </c>
       <c r="L61" s="40">
-        <f t="shared" ref="L61:L62" si="18">K61*5</f>
+        <f t="shared" ref="L61:L62" si="17">K61*5</f>
         <v>5</v>
       </c>
-      <c r="M61" s="73" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="62" spans="1:13">
+      <c r="M61" s="39"/>
+      <c r="O61" s="87"/>
+    </row>
+    <row r="62" spans="1:15" ht="24">
       <c r="A62" s="2"/>
       <c r="B62" s="34">
         <f t="shared" si="0"/>
         <v>53</v>
       </c>
       <c r="C62" s="43" t="s">
-        <v>211</v>
+        <v>201</v>
       </c>
       <c r="D62" s="36" t="s">
-        <v>212</v>
+        <v>202</v>
       </c>
       <c r="E62" s="37" t="s">
-        <v>213</v>
+        <v>203</v>
       </c>
       <c r="F62" s="36" t="s">
-        <v>214</v>
+        <v>204</v>
       </c>
       <c r="G62" s="37" t="s">
-        <v>215</v>
+        <v>205</v>
       </c>
       <c r="H62" s="38" t="s">
-        <v>216</v>
+        <v>206</v>
       </c>
       <c r="I62" s="36" t="s">
         <v>53</v>
@@ -4134,12 +4224,15 @@
         <v>1</v>
       </c>
       <c r="L62" s="37">
-        <f t="shared" si="18"/>
+        <f t="shared" si="17"/>
         <v>5</v>
       </c>
-      <c r="M62" s="36"/>
-    </row>
-    <row r="63" spans="1:13" ht="24">
+      <c r="M62" s="64" t="s">
+        <v>249</v>
+      </c>
+      <c r="O62" s="87"/>
+    </row>
+    <row r="63" spans="1:15" ht="36">
       <c r="A63" s="2"/>
       <c r="B63" s="34">
         <f t="shared" si="0"/>
@@ -4149,19 +4242,19 @@
         <v>201</v>
       </c>
       <c r="D63" s="39" t="s">
-        <v>217</v>
+        <v>207</v>
       </c>
       <c r="E63" s="40" t="s">
-        <v>218</v>
+        <v>208</v>
       </c>
       <c r="F63" s="39" t="s">
-        <v>219</v>
+        <v>209</v>
       </c>
       <c r="G63" s="40" t="s">
-        <v>220</v>
+        <v>210</v>
       </c>
       <c r="H63" s="41" t="s">
-        <v>221</v>
+        <v>206</v>
       </c>
       <c r="I63" s="36" t="s">
         <v>53</v>
@@ -4171,34 +4264,36 @@
         <v>1</v>
       </c>
       <c r="L63" s="40">
-        <f t="shared" ref="L63:L64" si="19">K63*5</f>
+        <f t="shared" ref="L63:L64" si="18">K63*5</f>
         <v>5</v>
       </c>
-      <c r="M63" s="39"/>
-    </row>
-    <row r="64" spans="1:13">
+      <c r="M63" s="64" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="64" spans="1:15">
       <c r="A64" s="2"/>
       <c r="B64" s="34">
         <f t="shared" si="0"/>
         <v>55</v>
       </c>
       <c r="C64" s="43" t="s">
-        <v>201</v>
+        <v>211</v>
       </c>
       <c r="D64" s="36" t="s">
-        <v>222</v>
+        <v>212</v>
       </c>
       <c r="E64" s="37" t="s">
-        <v>223</v>
+        <v>213</v>
       </c>
       <c r="F64" s="36" t="s">
-        <v>224</v>
+        <v>214</v>
       </c>
       <c r="G64" s="37" t="s">
-        <v>225</v>
+        <v>215</v>
       </c>
       <c r="H64" s="38" t="s">
-        <v>226</v>
+        <v>216</v>
       </c>
       <c r="I64" s="36" t="s">
         <v>53</v>
@@ -4208,12 +4303,12 @@
         <v>1</v>
       </c>
       <c r="L64" s="37">
-        <f t="shared" si="19"/>
+        <f t="shared" si="18"/>
         <v>5</v>
       </c>
       <c r="M64" s="36"/>
     </row>
-    <row r="65" spans="1:13">
+    <row r="65" spans="1:13" ht="24">
       <c r="A65" s="2"/>
       <c r="B65" s="34">
         <f t="shared" si="0"/>
@@ -4223,19 +4318,19 @@
         <v>201</v>
       </c>
       <c r="D65" s="39" t="s">
-        <v>227</v>
+        <v>217</v>
       </c>
       <c r="E65" s="40" t="s">
-        <v>228</v>
+        <v>218</v>
       </c>
       <c r="F65" s="39" t="s">
-        <v>229</v>
+        <v>219</v>
       </c>
       <c r="G65" s="40" t="s">
-        <v>230</v>
+        <v>220</v>
       </c>
       <c r="H65" s="41" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
       <c r="I65" s="36" t="s">
         <v>53</v>
@@ -4245,7 +4340,7 @@
         <v>1</v>
       </c>
       <c r="L65" s="40">
-        <f t="shared" ref="L65:L71" si="20">K65*5</f>
+        <f t="shared" ref="L65:L66" si="19">K65*5</f>
         <v>5</v>
       </c>
       <c r="M65" s="39"/>
@@ -4256,167 +4351,168 @@
         <f t="shared" si="0"/>
         <v>57</v>
       </c>
-      <c r="C66" s="35" t="s">
+      <c r="C66" s="43" t="s">
+        <v>201</v>
+      </c>
+      <c r="D66" s="36" t="s">
+        <v>222</v>
+      </c>
+      <c r="E66" s="37" t="s">
+        <v>223</v>
+      </c>
+      <c r="F66" s="36" t="s">
+        <v>224</v>
+      </c>
+      <c r="G66" s="37" t="s">
+        <v>225</v>
+      </c>
+      <c r="H66" s="38" t="s">
+        <v>226</v>
+      </c>
+      <c r="I66" s="36" t="s">
+        <v>53</v>
+      </c>
+      <c r="J66" s="36"/>
+      <c r="K66" s="56">
+        <v>1</v>
+      </c>
+      <c r="L66" s="37">
+        <f t="shared" si="19"/>
+        <v>5</v>
+      </c>
+      <c r="M66" s="36"/>
+    </row>
+    <row r="67" spans="1:13">
+      <c r="A67" s="2"/>
+      <c r="B67" s="34">
+        <f t="shared" si="0"/>
+        <v>58</v>
+      </c>
+      <c r="C67" s="35" t="s">
+        <v>201</v>
+      </c>
+      <c r="D67" s="39" t="s">
+        <v>227</v>
+      </c>
+      <c r="E67" s="40" t="s">
+        <v>228</v>
+      </c>
+      <c r="F67" s="39" t="s">
+        <v>229</v>
+      </c>
+      <c r="G67" s="40" t="s">
+        <v>230</v>
+      </c>
+      <c r="H67" s="41" t="s">
+        <v>226</v>
+      </c>
+      <c r="I67" s="36" t="s">
+        <v>53</v>
+      </c>
+      <c r="J67" s="36"/>
+      <c r="K67" s="57">
+        <v>1</v>
+      </c>
+      <c r="L67" s="40">
+        <f t="shared" ref="L67:L73" si="20">K67*5</f>
+        <v>5</v>
+      </c>
+      <c r="M67" s="39"/>
+    </row>
+    <row r="68" spans="1:13">
+      <c r="A68" s="2"/>
+      <c r="B68" s="34">
+        <f t="shared" si="0"/>
+        <v>59</v>
+      </c>
+      <c r="C68" s="35" t="s">
         <v>231</v>
       </c>
-      <c r="D66" s="39" t="s">
+      <c r="D68" s="39" t="s">
         <v>232</v>
       </c>
-      <c r="E66" s="40" t="s">
+      <c r="E68" s="40" t="s">
         <v>233</v>
       </c>
-      <c r="F66" s="39" t="s">
+      <c r="F68" s="39" t="s">
         <v>53</v>
       </c>
-      <c r="G66" s="40" t="s">
+      <c r="G68" s="40" t="s">
         <v>234</v>
       </c>
-      <c r="H66" s="41"/>
-      <c r="I66" s="58"/>
-      <c r="J66" s="36"/>
-      <c r="K66" s="57">
+      <c r="H68" s="41"/>
+      <c r="I68" s="58"/>
+      <c r="J68" s="36"/>
+      <c r="K68" s="57">
         <v>1</v>
       </c>
-      <c r="L66" s="40">
+      <c r="L68" s="40">
         <f t="shared" si="20"/>
         <v>5</v>
       </c>
-      <c r="M66" s="39"/>
-    </row>
-    <row r="67" spans="1:13" ht="48">
-      <c r="A67" s="2"/>
-      <c r="B67" s="34">
-        <f t="shared" si="0"/>
-        <v>58</v>
-      </c>
-      <c r="C67" s="42" t="s">
+      <c r="M68" s="39"/>
+    </row>
+    <row r="69" spans="1:13" ht="48">
+      <c r="A69" s="2"/>
+      <c r="B69" s="34">
+        <f t="shared" si="0"/>
+        <v>60</v>
+      </c>
+      <c r="C69" s="42" t="s">
         <v>235</v>
       </c>
-      <c r="D67" s="39" t="s">
+      <c r="D69" s="39" t="s">
         <v>232</v>
       </c>
-      <c r="E67" s="40" t="s">
+      <c r="E69" s="40" t="s">
         <v>236</v>
       </c>
-      <c r="F67" s="39" t="s">
+      <c r="F69" s="39" t="s">
         <v>53</v>
       </c>
-      <c r="G67" s="39" t="s">
+      <c r="G69" s="39" t="s">
         <v>53</v>
       </c>
-      <c r="H67" s="40" t="s">
+      <c r="H69" s="40" t="s">
         <v>53</v>
       </c>
-      <c r="I67" s="36" t="s">
+      <c r="I69" s="36" t="s">
         <v>53</v>
       </c>
-      <c r="J67" s="59" t="s">
+      <c r="J69" s="59" t="s">
         <v>237</v>
       </c>
-      <c r="K67" s="57">
+      <c r="K69" s="57">
         <v>1</v>
       </c>
-      <c r="L67" s="40">
+      <c r="L69" s="40">
         <f t="shared" si="20"/>
         <v>5</v>
       </c>
-      <c r="M67" s="39"/>
-    </row>
-    <row r="68" spans="1:13" ht="48.75" thickBot="1">
-      <c r="A68" s="2"/>
-      <c r="B68" s="34">
-        <f t="shared" si="0"/>
-        <v>59</v>
-      </c>
-      <c r="C68" s="35" t="s">
-        <v>238</v>
-      </c>
-      <c r="D68" s="39" t="s">
-        <v>232</v>
-      </c>
-      <c r="E68" s="40" t="s">
-        <v>239</v>
-      </c>
-      <c r="F68" s="39" t="s">
-        <v>53</v>
-      </c>
-      <c r="G68" s="40" t="s">
-        <v>53</v>
-      </c>
-      <c r="H68" s="41" t="s">
-        <v>53</v>
-      </c>
-      <c r="I68" s="36" t="s">
-        <v>53</v>
-      </c>
-      <c r="J68" s="59" t="s">
-        <v>237</v>
-      </c>
-      <c r="K68" s="57">
-        <v>1</v>
-      </c>
-      <c r="L68" s="40">
-        <v>1</v>
-      </c>
-      <c r="M68" s="39"/>
-    </row>
-    <row r="69" spans="1:13" ht="24.75" thickBot="1">
-      <c r="A69" s="2"/>
-      <c r="B69" s="34">
-        <f t="shared" si="0"/>
-        <v>60</v>
-      </c>
-      <c r="C69" s="66" t="s">
-        <v>240</v>
-      </c>
-      <c r="D69" s="69" t="s">
-        <v>232</v>
-      </c>
-      <c r="E69" s="40" t="s">
-        <v>241</v>
-      </c>
-      <c r="F69" s="39" t="s">
-        <v>53</v>
-      </c>
-      <c r="G69" s="40" t="s">
-        <v>244</v>
-      </c>
-      <c r="H69" s="39" t="s">
-        <v>53</v>
-      </c>
-      <c r="I69" s="36" t="s">
-        <v>53</v>
-      </c>
-      <c r="J69" s="59" t="s">
-        <v>237</v>
-      </c>
-      <c r="K69" s="36">
-        <v>3</v>
-      </c>
-      <c r="L69" s="40">
-        <f t="shared" si="20"/>
-        <v>15</v>
-      </c>
       <c r="M69" s="39"/>
     </row>
-    <row r="70" spans="1:13" ht="24.75" thickBot="1">
+    <row r="70" spans="1:13" ht="48.75" thickBot="1">
       <c r="A70" s="2"/>
       <c r="B70" s="34">
         <f t="shared" si="0"/>
         <v>61</v>
       </c>
-      <c r="C70" s="67"/>
-      <c r="D70" s="70"/>
+      <c r="C70" s="35" t="s">
+        <v>238</v>
+      </c>
+      <c r="D70" s="39" t="s">
+        <v>232</v>
+      </c>
       <c r="E70" s="40" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="F70" s="39" t="s">
         <v>53</v>
       </c>
       <c r="G70" s="40" t="s">
-        <v>245</v>
-      </c>
-      <c r="H70" s="39" t="s">
+        <v>53</v>
+      </c>
+      <c r="H70" s="41" t="s">
         <v>53</v>
       </c>
       <c r="I70" s="36" t="s">
@@ -4425,12 +4521,11 @@
       <c r="J70" s="59" t="s">
         <v>237</v>
       </c>
-      <c r="K70" s="36">
-        <v>2</v>
+      <c r="K70" s="57">
+        <v>1</v>
       </c>
       <c r="L70" s="40">
-        <f t="shared" si="20"/>
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="M70" s="39"/>
     </row>
@@ -4440,16 +4535,20 @@
         <f t="shared" si="0"/>
         <v>62</v>
       </c>
-      <c r="C71" s="68"/>
-      <c r="D71" s="71"/>
+      <c r="C71" s="79" t="s">
+        <v>240</v>
+      </c>
+      <c r="D71" s="82" t="s">
+        <v>232</v>
+      </c>
       <c r="E71" s="40" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="F71" s="39" t="s">
         <v>53</v>
       </c>
       <c r="G71" s="40" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="H71" s="39" t="s">
         <v>53</v>
@@ -4461,57 +4560,127 @@
         <v>237</v>
       </c>
       <c r="K71" s="36">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L71" s="40">
         <f t="shared" si="20"/>
+        <v>15</v>
+      </c>
+      <c r="M71" s="39"/>
+    </row>
+    <row r="72" spans="1:13" ht="24.75" thickBot="1">
+      <c r="A72" s="2"/>
+      <c r="B72" s="34">
+        <f t="shared" si="0"/>
+        <v>63</v>
+      </c>
+      <c r="C72" s="80"/>
+      <c r="D72" s="83"/>
+      <c r="E72" s="40" t="s">
+        <v>242</v>
+      </c>
+      <c r="F72" s="39" t="s">
+        <v>53</v>
+      </c>
+      <c r="G72" s="40" t="s">
+        <v>245</v>
+      </c>
+      <c r="H72" s="39" t="s">
+        <v>53</v>
+      </c>
+      <c r="I72" s="36" t="s">
+        <v>53</v>
+      </c>
+      <c r="J72" s="59" t="s">
+        <v>237</v>
+      </c>
+      <c r="K72" s="36">
+        <v>2</v>
+      </c>
+      <c r="L72" s="40">
+        <f t="shared" si="20"/>
+        <v>10</v>
+      </c>
+      <c r="M72" s="39"/>
+    </row>
+    <row r="73" spans="1:13" ht="24.75" thickBot="1">
+      <c r="A73" s="2"/>
+      <c r="B73" s="34">
+        <f t="shared" si="0"/>
+        <v>64</v>
+      </c>
+      <c r="C73" s="81"/>
+      <c r="D73" s="84"/>
+      <c r="E73" s="40" t="s">
+        <v>243</v>
+      </c>
+      <c r="F73" s="39" t="s">
+        <v>53</v>
+      </c>
+      <c r="G73" s="40" t="s">
+        <v>246</v>
+      </c>
+      <c r="H73" s="39" t="s">
+        <v>53</v>
+      </c>
+      <c r="I73" s="36" t="s">
+        <v>53</v>
+      </c>
+      <c r="J73" s="59" t="s">
+        <v>237</v>
+      </c>
+      <c r="K73" s="36">
+        <v>4</v>
+      </c>
+      <c r="L73" s="40">
+        <f t="shared" si="20"/>
         <v>20</v>
       </c>
-      <c r="M71" s="39"/>
-    </row>
-    <row r="72" spans="1:13">
-      <c r="A72" s="2"/>
-      <c r="B72" s="44"/>
-      <c r="C72" s="45"/>
-      <c r="D72" s="46"/>
-      <c r="E72" s="47"/>
-      <c r="F72" s="48"/>
-      <c r="G72" s="49"/>
-      <c r="H72" s="48"/>
-      <c r="I72" s="49"/>
-      <c r="J72" s="49"/>
-      <c r="K72" s="49"/>
-      <c r="L72" s="49"/>
-      <c r="M72" s="60"/>
-    </row>
-    <row r="73" spans="1:13">
-      <c r="A73" s="2"/>
-      <c r="B73" s="50"/>
-      <c r="C73" s="51"/>
-      <c r="D73" s="52"/>
-      <c r="E73" s="53"/>
-      <c r="F73" s="53"/>
-      <c r="G73" s="53"/>
-      <c r="H73" s="53"/>
-      <c r="I73" s="53"/>
-      <c r="J73" s="53"/>
-      <c r="K73" s="53"/>
-      <c r="L73" s="53"/>
-      <c r="M73" s="61"/>
+      <c r="M73" s="39"/>
+    </row>
+    <row r="74" spans="1:13">
+      <c r="A74" s="2"/>
+      <c r="B74" s="44"/>
+      <c r="C74" s="45"/>
+      <c r="D74" s="46"/>
+      <c r="E74" s="47"/>
+      <c r="F74" s="48"/>
+      <c r="G74" s="49"/>
+      <c r="H74" s="48"/>
+      <c r="I74" s="49"/>
+      <c r="J74" s="49"/>
+      <c r="K74" s="49"/>
+      <c r="L74" s="49"/>
+      <c r="M74" s="60"/>
+    </row>
+    <row r="75" spans="1:13">
+      <c r="A75" s="2"/>
+      <c r="B75" s="50"/>
+      <c r="C75" s="51"/>
+      <c r="D75" s="52"/>
+      <c r="E75" s="53"/>
+      <c r="F75" s="53"/>
+      <c r="G75" s="53"/>
+      <c r="H75" s="53"/>
+      <c r="I75" s="53"/>
+      <c r="J75" s="53"/>
+      <c r="K75" s="53"/>
+      <c r="L75" s="53"/>
+      <c r="M75" s="61"/>
     </row>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="I1:M1"/>
     <mergeCell ref="M3:M8"/>
-    <mergeCell ref="C69:C71"/>
-    <mergeCell ref="D69:D71"/>
+    <mergeCell ref="C71:C73"/>
+    <mergeCell ref="D71:D73"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="J68" r:id="rId1"/>
-    <hyperlink ref="J67" r:id="rId2"/>
-    <hyperlink ref="J69" r:id="rId3"/>
-    <hyperlink ref="J70" r:id="rId4"/>
-    <hyperlink ref="J71" r:id="rId5"/>
+    <hyperlink ref="J70" r:id="rId1"/>
+    <hyperlink ref="J69" r:id="rId2"/>
+    <hyperlink ref="J71" r:id="rId3"/>
+    <hyperlink ref="J72" r:id="rId4"/>
+    <hyperlink ref="J73" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId6"/>

</xml_diff>